<commit_message>
Prefer evaluator assignment titles in staff evaluations
</commit_message>
<xml_diff>
--- a/scripts/teacher-imports/assignments/inputs/teacher-assignments-import-5.xlsx
+++ b/scripts/teacher-imports/assignments/inputs/teacher-assignments-import-5.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\edu-affairs-v2\scripts\teacher-imports\assignments\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC17278A-A997-46EE-8EEB-EF0B6D4B970A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B4822E-CD57-4EE2-929C-037F91FA3BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12975" yWindow="2985" windowWidth="15645" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4215" yWindow="2250" windowWidth="20190" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="التوزيع" sheetId="1" r:id="rId1"/>
-    <sheet name="التوزيع (الفالح)" sheetId="4" r:id="rId2"/>
-    <sheet name="تعليمات" sheetId="2" r:id="rId3"/>
-    <sheet name="نسخة من التوزيع" sheetId="3" r:id="rId4"/>
-    <sheet name="التوزيع (2)" sheetId="5" r:id="rId5"/>
+    <sheet name="التوزيع (3)" sheetId="6" r:id="rId2"/>
+    <sheet name="التوزيع (الفالح)" sheetId="4" r:id="rId3"/>
+    <sheet name="تعليمات" sheetId="2" r:id="rId4"/>
+    <sheet name="نسخة من التوزيع" sheetId="3" r:id="rId5"/>
+    <sheet name="التوزيع (2)" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="299">
   <si>
     <t>الحقل</t>
   </si>
@@ -870,13 +871,64 @@
   </si>
   <si>
     <t>mrb-boys-sayh-g2-quran-1-arabic</t>
+  </si>
+  <si>
+    <t>w-a-atwala@qz.org.sa</t>
+  </si>
+  <si>
+    <t>mrb-girls</t>
+  </si>
+  <si>
+    <t>g5-quran-2</t>
+  </si>
+  <si>
+    <t>mrb-girls-g5-quran-2-tajweed</t>
+  </si>
+  <si>
+    <t>خامس تحفيظ أ</t>
+  </si>
+  <si>
+    <t>سادس عام</t>
+  </si>
+  <si>
+    <t>سادس تحفيظ</t>
+  </si>
+  <si>
+    <t>g5-quran-1</t>
+  </si>
+  <si>
+    <t>g6-quran-1</t>
+  </si>
+  <si>
+    <t>mrb-girls-g5-quran-1-tajweed</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-general-1-quran</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-general-1-pe</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-quran-1-quran</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-quran-1-tajweed</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-general-1-social-studies</t>
+  </si>
+  <si>
+    <t>mrb-girls-g6-quran-1-social-studies</t>
+  </si>
+  <si>
+    <t>خامس  تحفيظ  ب</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -887,8 +939,16 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="178"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -921,6 +981,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -931,10 +996,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -964,11 +1030,29 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -982,7 +1066,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TeacherAssignmentsImportTable" displayName="TeacherAssignmentsImportTable" ref="A1:J205">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TeacherAssignmentsImportTable" displayName="TeacherAssignmentsImportTable" ref="A1:J185">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="بريد المعلم"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="معرّف المدرسة"/>
@@ -991,7 +1075,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="معرّف الفصل"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="اسم الفصل للتوضيح"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="معرّف إسناد المادة"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="رمز المادة"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="رمز المادة" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="اسم المادة للتوضيح"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="حالة الإسناد"/>
   </tableColumns>
@@ -1000,6 +1084,24 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F8F6036A-DAED-41D6-AECB-D26F620EAABF}" name="TeacherAssignmentsImportTable6" displayName="TeacherAssignmentsImportTable6" ref="A1:J205">
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{49620D7E-8038-4A6F-8C05-4ADEAF44CE57}" name="بريد المعلم"/>
+    <tableColumn id="2" xr3:uid="{83DC1D65-67E9-4B73-802F-2A24C885202F}" name="معرّف المدرسة"/>
+    <tableColumn id="3" xr3:uid="{E37A54AC-AB6C-42EB-92FE-067B5C91E1F4}" name="معرّف السنة الدراسية"/>
+    <tableColumn id="4" xr3:uid="{D2D6E63E-2EDD-4B4C-A044-5F9A2AA9C284}" name="معرّف الفصل الدراسي"/>
+    <tableColumn id="5" xr3:uid="{112798F5-595C-4512-8EE1-327993142188}" name="معرّف الفصل"/>
+    <tableColumn id="6" xr3:uid="{E3E806E7-DD9C-4832-999E-6D03F5831094}" name="اسم الفصل للتوضيح"/>
+    <tableColumn id="7" xr3:uid="{409C4D6A-73EF-47D8-98A9-C8C13F51DA87}" name="معرّف إسناد المادة"/>
+    <tableColumn id="8" xr3:uid="{42A00B9F-21A8-4B34-928A-8B6876BD656F}" name="رمز المادة"/>
+    <tableColumn id="9" xr3:uid="{02544783-8720-4B1E-A520-A461E4BEFF17}" name="اسم المادة للتوضيح"/>
+    <tableColumn id="10" xr3:uid="{0EEFBBD6-F60E-4B81-B48F-2234C3DF8AFD}" name="حالة الإسناد"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A1F22050-3E2D-4D7E-BD84-34E8028A1739}" name="TeacherAssignmentsImportTable4" displayName="TeacherAssignmentsImportTable4" ref="A1:J307">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{FFCD2B81-D0EC-4759-829E-4620D681AF09}" name="بريد المعلم"/>
@@ -1017,7 +1119,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="TeacherAssignmentsImportTable3" displayName="TeacherAssignmentsImportTable3" ref="A1:J307">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="بريد المعلم"/>
@@ -1035,7 +1137,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D49BE05C-90B1-42A0-B5E7-D768F1CDAAC0}" name="TeacherAssignmentsImportTable5" displayName="TeacherAssignmentsImportTable5" ref="A1:J307">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{2D3F7724-E3BE-4AC8-9EAF-33DD236D8A8A}" name="بريد المعلم"/>
@@ -1202,6 +1304,325 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="19.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.375" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.125" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>284</v>
+      </c>
+      <c r="F2" t="s">
+        <v>298</v>
+      </c>
+      <c r="G2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="I2" t="s">
+        <v>126</v>
+      </c>
+      <c r="J2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="G3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="I3" t="s">
+        <v>126</v>
+      </c>
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="13" customFormat="1" ht="15">
+      <c r="A4" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>282</v>
+      </c>
+      <c r="B5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="G5" t="s">
+        <v>296</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>282</v>
+      </c>
+      <c r="B6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="G6" t="s">
+        <v>293</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="13" customFormat="1" ht="15">
+      <c r="A7" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>282</v>
+      </c>
+      <c r="B8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
+        <v>290</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G8" t="s">
+        <v>295</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="I8" t="s">
+        <v>126</v>
+      </c>
+      <c r="J8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>282</v>
+      </c>
+      <c r="B9" t="s">
+        <v>283</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G9" t="s">
+        <v>297</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="J2:J279" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"ACTIVE,INACTIVE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8BCF69B-267E-4586-9F72-B180F18F54F5}">
   <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -1571,7 +1992,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="J2:J299" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="J2:J299" xr:uid="{199E722F-C52E-4C1B-8672-FB0DD5507C1E}">
       <formula1>"ACTIVE,INACTIVE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1582,7 +2003,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{855DE344-A4BF-4E86-B1DC-478DCAD9707B}">
   <dimension ref="A1:J66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -3723,7 +4144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -3833,7 +4254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -5974,7 +6395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{029718D0-2D8E-4FBD-8D78-A36ECF33734C}">
   <dimension ref="A1:J101"/>
   <sheetFormatPr defaultRowHeight="14.25"/>

</xml_diff>